<commit_message>
some changes in statuses
</commit_message>
<xml_diff>
--- a/burocracy/final_docs/учет бумажек.xlsx
+++ b/burocracy/final_docs/учет бумажек.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\disser\burocracy\final_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C077B47-FECF-482B-82C7-2BD7C3E8C47E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E83063-E8AB-4C2E-B556-B4D301057CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{134430FC-25E2-4572-9815-FE2A91FBD179}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
   <si>
     <t>Имя</t>
   </si>
@@ -146,9 +146,6 @@
     <t>МИФИ</t>
   </si>
   <si>
-    <t>20.10 отправил в тг Надежде проект заключения</t>
-  </si>
-  <si>
     <t>согласен на 11.12 11:00?</t>
   </si>
   <si>
@@ -161,10 +158,49 @@
     <t>andreev_stepan@mail.ru</t>
   </si>
   <si>
-    <t>20.10.26 драфт отзыва отправил себе вк</t>
-  </si>
-  <si>
     <t>21.10.26 отправил диссер и автореферат</t>
+  </si>
+  <si>
+    <t>Корреспонденция</t>
+  </si>
+  <si>
+    <t>Куда</t>
+  </si>
+  <si>
+    <t>Автореферат</t>
+  </si>
+  <si>
+    <t>Диссер</t>
+  </si>
+  <si>
+    <t>ТАСС</t>
+  </si>
+  <si>
+    <t>готово?</t>
+  </si>
+  <si>
+    <t>МФТИ</t>
+  </si>
+  <si>
+    <t>Лактионову</t>
+  </si>
+  <si>
+    <t>Минцифры</t>
+  </si>
+  <si>
+    <t>РГБ</t>
+  </si>
+  <si>
+    <t>РГБ или Лактионову</t>
+  </si>
+  <si>
+    <t>22.10 Надежда сказала что передала</t>
+  </si>
+  <si>
+    <t>23/10/26 передал заверенній оригинал в 506</t>
+  </si>
+  <si>
+    <t>диссовет</t>
   </si>
 </sst>
 </file>
@@ -313,7 +349,119 @@
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="23">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -673,7 +821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3A0C460-2CFB-4414-A3CC-DFB3884CADAE}">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" style="4" hidden="1" customWidth="1"/>
@@ -710,7 +858,7 @@
         <v>2</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>34</v>
@@ -786,10 +934,10 @@
         <v>1</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="I3" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>21</v>
@@ -819,16 +967,16 @@
         <v>26</v>
       </c>
       <c r="G4" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I4" s="6">
         <v>0</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
@@ -858,7 +1006,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I5" s="2">
         <v>0</v>
@@ -930,7 +1078,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I7" s="9">
         <v>0</v>
@@ -949,7 +1097,7 @@
       </c>
       <c r="G8" s="12"/>
       <c r="H8" s="11" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="I8" s="2">
         <v>0</v>
@@ -957,18 +1105,144 @@
     </row>
     <row r="9" spans="1:14" customFormat="1" x14ac:dyDescent="0.3">
       <c r="D9" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="13" t="s">
-        <v>40</v>
-      </c>
       <c r="G9" s="9">
         <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="E14" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="4">
+        <v>9</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="E15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="4">
+        <v>2</v>
+      </c>
+      <c r="G15" s="4">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="4">
+        <v>1</v>
+      </c>
+      <c r="G16" s="4">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="5:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E17" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="4">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="4">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="5:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E19" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F20" s="4">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4">
+        <v>1</v>
+      </c>
+      <c r="H20" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E21" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="4">
+        <v>6</v>
+      </c>
+      <c r="G21" s="4">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I8">
-    <cfRule type="colorScale" priority="13">
+    <cfRule type="colorScale" priority="41">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -980,20 +1254,20 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I7">
-    <cfRule type="cellIs" dxfId="6" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="40" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I8">
-    <cfRule type="cellIs" dxfId="5" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="39" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I8">
-    <cfRule type="cellIs" dxfId="4" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="44" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="45">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1005,7 +1279,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G7">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="35">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1017,15 +1291,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G7">
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="34" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G7">
-    <cfRule type="cellIs" dxfId="2" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="36" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="9">
+    <cfRule type="colorScale" priority="37">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1037,6 +1311,230 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="cellIs" dxfId="17" priority="29" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="cellIs" dxfId="16" priority="31" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H14:H15">
+    <cfRule type="cellIs" dxfId="15" priority="25" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="cellIs" dxfId="14" priority="21" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="cellIs" dxfId="13" priority="23" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="cellIs" dxfId="12" priority="17" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="cellIs" dxfId="11" priority="19" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
+    <cfRule type="cellIs" dxfId="10" priority="13" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
+    <cfRule type="cellIs" dxfId="9" priority="15" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H14:H15">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H14:H15">
+    <cfRule type="cellIs" dxfId="4" priority="47" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H21">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1048,12 +1546,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
+  <conditionalFormatting sqref="H21">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
+  <conditionalFormatting sqref="H21">
     <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>1</formula>
     </cfRule>

</xml_diff>